<commit_message>
feat: implement ScoreboardController and add initial team data assets
</commit_message>
<xml_diff>
--- a/excel/VAR 38+.xlsx
+++ b/excel/VAR 38+.xlsx
@@ -109,11 +109,11 @@
     <t>https://opknice.github.io/projectvar/allscore_var.html</t>
   </si>
   <si>
-    <t>นัดที่ 3</t>
-  </si>
-  <si>
     <t>VAR SUPER LEAUGE 38+
 🔴 https://www.youtube.com/@ViewtanArena/streams</t>
+  </si>
+  <si>
+    <t>นัดที่ 5</t>
   </si>
 </sst>
 </file>
@@ -648,16 +648,16 @@
         <v>16</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E2" s="32" t="s">
         <v>29</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -665,19 +665,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="D3" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E3" s="32" t="s">
         <v>29</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -685,19 +685,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E4" s="32" t="s">
         <v>29</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:6">

</xml_diff>